<commit_message>
convolution operators refactored, seem to work, not entirely sure yet
</commit_message>
<xml_diff>
--- a/src/test/filter-edge-sobel/proof_sobel_is_correct_small_line_gray.xlsx
+++ b/src/test/filter-edge-sobel/proof_sobel_is_correct_small_line_gray.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\cv-workbench\src\test\filter-edge-sobel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC365B3-B1D1-4843-8229-4B61167C7849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87801E85-19E8-41CA-8663-26176CF2D74A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="4880" windowWidth="16360" windowHeight="4980" xr2:uid="{FD9AEBEA-5D56-4DB4-9FDD-49E0E1A99388}"/>
+    <workbookView xWindow="-22350" yWindow="2280" windowWidth="16095" windowHeight="10695" activeTab="1" xr2:uid="{FD9AEBEA-5D56-4DB4-9FDD-49E0E1A99388}"/>
   </bookViews>
   <sheets>
     <sheet name="small_line_gray" sheetId="1" r:id="rId1"/>
-    <sheet name="sep_row" sheetId="2" r:id="rId2"/>
-    <sheet name="sep_col" sheetId="3" r:id="rId3"/>
-    <sheet name="sep_row_col" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
+    <sheet name="sep_row" sheetId="2" r:id="rId3"/>
+    <sheet name="sep_col" sheetId="3" r:id="rId4"/>
+    <sheet name="sep_row_col" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -104,7 +105,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1109,12 +1110,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AN67"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="12" max="21" width="5.6328125" customWidth="1"/>
+    <col min="12" max="21" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40">
+    <row r="1" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:40">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -1194,7 +1195,7 @@
       </c>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:40">
+    <row r="3" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1256,7 +1257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:40">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -1315,7 +1316,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:40">
+    <row r="5" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -1368,7 +1369,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:40">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -1409,7 +1410,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:40">
+    <row r="7" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -1456,7 +1457,7 @@
       <c r="X7" s="10"/>
       <c r="Y7" s="10"/>
     </row>
-    <row r="8" spans="1:40">
+    <row r="8" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -1503,7 +1504,7 @@
       <c r="X8" s="10"/>
       <c r="Y8" s="10"/>
     </row>
-    <row r="9" spans="1:40">
+    <row r="9" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -1548,7 +1549,7 @@
       <c r="X9" s="10"/>
       <c r="Y9" s="10"/>
     </row>
-    <row r="10" spans="1:40">
+    <row r="10" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -1613,7 +1614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:40">
+    <row r="11" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -1678,7 +1679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:40">
+    <row r="12" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -1734,7 +1735,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="14" spans="1:40">
+    <row r="14" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1742,7 +1743,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:40">
+    <row r="15" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -1852,7 +1853,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:40">
+    <row r="16" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>0</v>
       </c>
@@ -1962,7 +1963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:40">
+    <row r="17" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>1</v>
       </c>
@@ -2081,7 +2082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:40">
+    <row r="18" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>2</v>
       </c>
@@ -2200,7 +2201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:40">
+    <row r="19" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>3</v>
       </c>
@@ -2319,7 +2320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:40">
+    <row r="20" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>4</v>
       </c>
@@ -2438,7 +2439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:40">
+    <row r="21" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>5</v>
       </c>
@@ -2557,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:40">
+    <row r="22" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>6</v>
       </c>
@@ -2676,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:40">
+    <row r="23" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>7</v>
       </c>
@@ -2795,7 +2796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:40">
+    <row r="24" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>8</v>
       </c>
@@ -2914,7 +2915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:40">
+    <row r="25" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>9</v>
       </c>
@@ -3036,7 +3037,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:40">
+    <row r="26" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>10</v>
       </c>
@@ -3149,7 +3150,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:40">
+    <row r="28" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>1</v>
       </c>
@@ -3199,7 +3200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:40">
+    <row r="29" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -3309,7 +3310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:40">
+    <row r="30" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>0</v>
       </c>
@@ -3422,7 +3423,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:40">
+    <row r="31" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>1</v>
       </c>
@@ -3547,7 +3548,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:40">
+    <row r="32" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>2</v>
       </c>
@@ -3669,7 +3670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:38">
+    <row r="33" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>3</v>
       </c>
@@ -3791,7 +3792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:38">
+    <row r="34" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>4</v>
       </c>
@@ -3910,7 +3911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:38">
+    <row r="35" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>5</v>
       </c>
@@ -4029,7 +4030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:38">
+    <row r="36" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>6</v>
       </c>
@@ -4148,7 +4149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:38">
+    <row r="37" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>7</v>
       </c>
@@ -4267,7 +4268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:38">
+    <row r="38" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>8</v>
       </c>
@@ -4386,7 +4387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:38">
+    <row r="39" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>9</v>
       </c>
@@ -4505,7 +4506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:38">
+    <row r="40" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>10</v>
       </c>
@@ -4582,7 +4583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:38">
+    <row r="42" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>0</v>
       </c>
@@ -4605,7 +4606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:38">
+    <row r="43" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -4676,7 +4677,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:38">
+    <row r="44" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>0</v>
       </c>
@@ -4684,39 +4685,39 @@
         <v>0</v>
       </c>
       <c r="C44" s="7">
-        <f>B2+2*C2+D2</f>
+        <f t="shared" ref="C44:K44" si="21">B2+2*C2+D2</f>
         <v>11</v>
       </c>
       <c r="D44">
-        <f>C2+2*D2+E2</f>
+        <f t="shared" si="21"/>
         <v>4</v>
       </c>
       <c r="E44">
-        <f>D2+2*E2+F2</f>
+        <f t="shared" si="21"/>
         <v>9</v>
       </c>
       <c r="F44">
-        <f>E2+2*F2+G2</f>
+        <f t="shared" si="21"/>
         <v>258</v>
       </c>
       <c r="G44">
-        <f>F2+2*G2+H2</f>
+        <f t="shared" si="21"/>
         <v>520</v>
       </c>
       <c r="H44">
-        <f>G2+2*H2+I2</f>
+        <f t="shared" si="21"/>
         <v>328</v>
       </c>
       <c r="I44">
-        <f>H2+2*I2+J2</f>
+        <f t="shared" si="21"/>
         <v>186</v>
       </c>
       <c r="J44">
-        <f>I2+2*J2+K2</f>
+        <f t="shared" si="21"/>
         <v>283</v>
       </c>
       <c r="K44">
-        <f>J2+2*K2+L2</f>
+        <f t="shared" si="21"/>
         <v>316</v>
       </c>
       <c r="L44">
@@ -4759,7 +4760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:38">
+    <row r="45" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>1</v>
       </c>
@@ -4767,39 +4768,39 @@
         <v>0</v>
       </c>
       <c r="C45" s="7">
-        <f>B3+2*C3+D3</f>
+        <f t="shared" ref="C45:K45" si="22">B3+2*C3+D3</f>
         <v>2</v>
       </c>
       <c r="D45">
-        <f>C3+2*D3+E3</f>
+        <f t="shared" si="22"/>
         <v>5</v>
       </c>
       <c r="E45">
-        <f>D3+2*E3+F3</f>
+        <f t="shared" si="22"/>
         <v>4</v>
       </c>
       <c r="F45">
-        <f>E3+2*F3+G3</f>
+        <f t="shared" si="22"/>
         <v>256</v>
       </c>
       <c r="G45">
-        <f>F3+2*G3+H3</f>
+        <f t="shared" si="22"/>
         <v>510</v>
       </c>
       <c r="H45">
-        <f>G3+2*H3+I3</f>
+        <f t="shared" si="22"/>
         <v>258</v>
       </c>
       <c r="I45">
-        <f>H3+2*I3+J3</f>
+        <f t="shared" si="22"/>
         <v>16</v>
       </c>
       <c r="J45">
-        <f>I3+2*J3+K3</f>
+        <f t="shared" si="22"/>
         <v>33</v>
       </c>
       <c r="K45">
-        <f>J3+2*K3+L3</f>
+        <f t="shared" si="22"/>
         <v>40</v>
       </c>
       <c r="L45">
@@ -4842,7 +4843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:38">
+    <row r="46" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>2</v>
       </c>
@@ -4850,39 +4851,39 @@
         <v>0</v>
       </c>
       <c r="C46" s="7">
-        <f>B4+2*C4+D4</f>
+        <f t="shared" ref="C46:K46" si="23">B4+2*C4+D4</f>
         <v>8</v>
       </c>
       <c r="D46">
-        <f>C4+2*D4+E4</f>
+        <f t="shared" si="23"/>
         <v>4</v>
       </c>
       <c r="E46">
-        <f>D4+2*E4+F4</f>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="F46">
-        <f>E4+2*F4+G4</f>
+        <f t="shared" si="23"/>
         <v>255</v>
       </c>
       <c r="G46">
-        <f>F4+2*G4+H4</f>
+        <f t="shared" si="23"/>
         <v>510</v>
       </c>
       <c r="H46">
-        <f>G4+2*H4+I4</f>
+        <f t="shared" si="23"/>
         <v>255</v>
       </c>
       <c r="I46">
-        <f>H4+2*I4+J4</f>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="J46">
-        <f>I4+2*J4+K4</f>
+        <f t="shared" si="23"/>
         <v>3</v>
       </c>
       <c r="K46">
-        <f>J4+2*K4+L4</f>
+        <f t="shared" si="23"/>
         <v>4</v>
       </c>
       <c r="L46">
@@ -4925,7 +4926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:38">
+    <row r="47" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>3</v>
       </c>
@@ -4933,39 +4934,39 @@
         <v>0</v>
       </c>
       <c r="C47">
-        <f>B5+2*C5+D5</f>
+        <f t="shared" ref="C47:K47" si="24">B5+2*C5+D5</f>
         <v>0</v>
       </c>
       <c r="D47">
-        <f>C5+2*D5+E5</f>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
       <c r="E47">
-        <f>D5+2*E5+F5</f>
+        <f t="shared" si="24"/>
         <v>3</v>
       </c>
       <c r="F47">
-        <f>E5+2*F5+G5</f>
+        <f t="shared" si="24"/>
         <v>258</v>
       </c>
       <c r="G47">
-        <f>F5+2*G5+H5</f>
+        <f t="shared" si="24"/>
         <v>511</v>
       </c>
       <c r="H47">
-        <f>G5+2*H5+I5</f>
+        <f t="shared" si="24"/>
         <v>258</v>
       </c>
       <c r="I47">
-        <f>H5+2*I5+J5</f>
+        <f t="shared" si="24"/>
         <v>6</v>
       </c>
       <c r="J47">
-        <f>I5+2*J5+K5</f>
+        <f t="shared" si="24"/>
         <v>3</v>
       </c>
       <c r="K47">
-        <f>J5+2*K5+L5</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="L47">
@@ -5008,7 +5009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:38">
+    <row r="48" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>4</v>
       </c>
@@ -5016,39 +5017,39 @@
         <v>0</v>
       </c>
       <c r="C48">
-        <f>B6+2*C6+D6</f>
+        <f t="shared" ref="C48:K48" si="25">B6+2*C6+D6</f>
         <v>3</v>
       </c>
       <c r="D48">
-        <f>C6+2*D6+E6</f>
+        <f t="shared" si="25"/>
         <v>6</v>
       </c>
       <c r="E48">
-        <f>D6+2*E6+F6</f>
+        <f t="shared" si="25"/>
         <v>3</v>
       </c>
       <c r="F48">
-        <f>E6+2*F6+G6</f>
+        <f t="shared" si="25"/>
         <v>255</v>
       </c>
       <c r="G48">
-        <f>F6+2*G6+H6</f>
+        <f t="shared" si="25"/>
         <v>510</v>
       </c>
       <c r="H48">
-        <f>G6+2*H6+I6</f>
+        <f t="shared" si="25"/>
         <v>255</v>
       </c>
       <c r="I48">
-        <f>H6+2*I6+J6</f>
+        <f t="shared" si="25"/>
         <v>1</v>
       </c>
       <c r="J48">
-        <f>I6+2*J6+K6</f>
+        <f t="shared" si="25"/>
         <v>3</v>
       </c>
       <c r="K48">
-        <f>J6+2*K6+L6</f>
+        <f t="shared" si="25"/>
         <v>4</v>
       </c>
       <c r="L48">
@@ -5091,7 +5092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:26">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>5</v>
       </c>
@@ -5099,39 +5100,39 @@
         <v>0</v>
       </c>
       <c r="C49">
-        <f>B7+2*C7+D7</f>
+        <f t="shared" ref="C49:K49" si="26">B7+2*C7+D7</f>
         <v>10</v>
       </c>
       <c r="D49">
-        <f>C7+2*D7+E7</f>
+        <f t="shared" si="26"/>
         <v>5</v>
       </c>
       <c r="E49">
-        <f>D7+2*E7+F7</f>
+        <f t="shared" si="26"/>
         <v>1</v>
       </c>
       <c r="F49">
-        <f>E7+2*F7+G7</f>
+        <f t="shared" si="26"/>
         <v>255</v>
       </c>
       <c r="G49">
-        <f>F7+2*G7+H7</f>
+        <f t="shared" si="26"/>
         <v>512</v>
       </c>
       <c r="H49">
-        <f>G7+2*H7+I7</f>
+        <f t="shared" si="26"/>
         <v>259</v>
       </c>
       <c r="I49">
-        <f>H7+2*I7+J7</f>
+        <f t="shared" si="26"/>
         <v>2</v>
       </c>
       <c r="J49">
-        <f>I7+2*J7+K7</f>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="K49">
-        <f>J7+2*K7+L7</f>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L49">
@@ -5174,7 +5175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:26">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
         <v>6</v>
       </c>
@@ -5182,39 +5183,39 @@
         <v>0</v>
       </c>
       <c r="C50">
-        <f>B8+2*C8+D8</f>
+        <f t="shared" ref="C50:K50" si="27">B8+2*C8+D8</f>
         <v>0</v>
       </c>
       <c r="D50">
-        <f>C8+2*D8+E8</f>
+        <f t="shared" si="27"/>
         <v>1</v>
       </c>
       <c r="E50">
-        <f>D8+2*E8+F8</f>
+        <f t="shared" si="27"/>
         <v>4</v>
       </c>
       <c r="F50">
-        <f>E8+2*F8+G8</f>
+        <f t="shared" si="27"/>
         <v>260</v>
       </c>
       <c r="G50">
-        <f>F8+2*G8+H8</f>
+        <f t="shared" si="27"/>
         <v>512</v>
       </c>
       <c r="H50">
-        <f>G8+2*H8+I8</f>
+        <f t="shared" si="27"/>
         <v>255</v>
       </c>
       <c r="I50">
-        <f>H8+2*I8+J8</f>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="J50">
-        <f>I8+2*J8+K8</f>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="K50">
-        <f>J8+2*K8+L8</f>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="L50">
@@ -5257,7 +5258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:26">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
         <v>7</v>
       </c>
@@ -5265,39 +5266,39 @@
         <v>0</v>
       </c>
       <c r="C51">
-        <f>B9+2*C9+D9</f>
+        <f t="shared" ref="C51:K51" si="28">B9+2*C9+D9</f>
         <v>1</v>
       </c>
       <c r="D51">
-        <f>C9+2*D9+E9</f>
+        <f t="shared" si="28"/>
         <v>3</v>
       </c>
       <c r="E51">
-        <f>D9+2*E9+F9</f>
+        <f t="shared" si="28"/>
         <v>3</v>
       </c>
       <c r="F51">
-        <f>E9+2*F9+G9</f>
+        <f t="shared" si="28"/>
         <v>256</v>
       </c>
       <c r="G51">
-        <f>F9+2*G9+H9</f>
+        <f t="shared" si="28"/>
         <v>510</v>
       </c>
       <c r="H51">
-        <f>G9+2*H9+I9</f>
+        <f t="shared" si="28"/>
         <v>256</v>
       </c>
       <c r="I51">
-        <f>H9+2*I9+J9</f>
+        <f t="shared" si="28"/>
         <v>2</v>
       </c>
       <c r="J51">
-        <f>I9+2*J9+K9</f>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
       <c r="K51">
-        <f>J9+2*K9+L9</f>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="L51">
@@ -5340,7 +5341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:26">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
         <v>8</v>
       </c>
@@ -5348,39 +5349,39 @@
         <v>0</v>
       </c>
       <c r="C52">
-        <f>B10+2*C10+D10</f>
+        <f t="shared" ref="C52:K52" si="29">B10+2*C10+D10</f>
         <v>1</v>
       </c>
       <c r="D52">
-        <f>C10+2*D10+E10</f>
+        <f t="shared" si="29"/>
         <v>3</v>
       </c>
       <c r="E52">
-        <f>D10+2*E10+F10</f>
+        <f t="shared" si="29"/>
         <v>6</v>
       </c>
       <c r="F52">
-        <f>E10+2*F10+G10</f>
+        <f t="shared" si="29"/>
         <v>255</v>
       </c>
       <c r="G52">
-        <f>F10+2*G10+H10</f>
+        <f t="shared" si="29"/>
         <v>507</v>
       </c>
       <c r="H52">
-        <f>G10+2*H10+I10</f>
+        <f t="shared" si="29"/>
         <v>259</v>
       </c>
       <c r="I52">
-        <f>H10+2*I10+J10</f>
+        <f t="shared" si="29"/>
         <v>5</v>
       </c>
       <c r="J52">
-        <f>I10+2*J10+K10</f>
+        <f t="shared" si="29"/>
         <v>1</v>
       </c>
       <c r="K52">
-        <f>J10+2*K10+L10</f>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="L52">
@@ -5423,7 +5424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:26">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
         <v>9</v>
       </c>
@@ -5431,39 +5432,39 @@
         <v>0</v>
       </c>
       <c r="C53">
-        <f>B11+2*C11+D11</f>
+        <f t="shared" ref="C53:K53" si="30">B11+2*C11+D11</f>
         <v>46</v>
       </c>
       <c r="D53">
-        <f>C11+2*D11+E11</f>
+        <f t="shared" si="30"/>
         <v>8</v>
       </c>
       <c r="E53">
-        <f>D11+2*E11+F11</f>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="F53">
-        <f>E11+2*F11+G11</f>
+        <f t="shared" si="30"/>
         <v>255</v>
       </c>
       <c r="G53">
-        <f>F11+2*G11+H11</f>
+        <f t="shared" si="30"/>
         <v>512</v>
       </c>
       <c r="H53">
-        <f>G11+2*H11+I11</f>
+        <f t="shared" si="30"/>
         <v>259</v>
       </c>
       <c r="I53">
-        <f>H11+2*I11+J11</f>
+        <f t="shared" si="30"/>
         <v>2</v>
       </c>
       <c r="J53">
-        <f>I11+2*J11+K11</f>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="K53">
-        <f>J11+2*K11+L11</f>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="L53">
@@ -5506,7 +5507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:26">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
         <v>10</v>
       </c>
@@ -5514,39 +5515,39 @@
         <v>0</v>
       </c>
       <c r="C54">
-        <f>B12+2*C12+D12</f>
+        <f t="shared" ref="C54:K54" si="31">B12+2*C12+D12</f>
         <v>146</v>
       </c>
       <c r="D54">
-        <f>C12+2*D12+E12</f>
+        <f t="shared" si="31"/>
         <v>34</v>
       </c>
       <c r="E54">
-        <f>D12+2*E12+F12</f>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="F54">
-        <f>E12+2*F12+G12</f>
+        <f t="shared" si="31"/>
         <v>254</v>
       </c>
       <c r="G54">
-        <f>F12+2*G12+H12</f>
+        <f t="shared" si="31"/>
         <v>509</v>
       </c>
       <c r="H54">
-        <f>G12+2*H12+I12</f>
+        <f t="shared" si="31"/>
         <v>256</v>
       </c>
       <c r="I54">
-        <f>H12+2*I12+J12</f>
+        <f t="shared" si="31"/>
         <v>1</v>
       </c>
       <c r="J54">
-        <f>I12+2*J12+K12</f>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="K54">
-        <f>J12+2*K12+L12</f>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="L54">
@@ -5589,7 +5590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:26">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>2</v>
       </c>
@@ -5598,31 +5599,31 @@
         <v>6</v>
       </c>
       <c r="D57">
-        <f t="shared" ref="D57:J57" si="21">C31+2*D31+E31</f>
+        <f t="shared" ref="D57:J57" si="32">C31+2*D31+E31</f>
         <v>11</v>
       </c>
       <c r="E57">
-        <f t="shared" si="21"/>
+        <f t="shared" si="32"/>
         <v>19</v>
       </c>
       <c r="F57">
-        <f t="shared" si="21"/>
+        <f t="shared" si="32"/>
         <v>24</v>
       </c>
       <c r="G57">
-        <f t="shared" si="21"/>
+        <f t="shared" si="32"/>
         <v>96</v>
       </c>
       <c r="H57">
-        <f t="shared" si="21"/>
+        <f t="shared" si="32"/>
         <v>341</v>
       </c>
       <c r="I57">
-        <f t="shared" si="21"/>
+        <f t="shared" si="32"/>
         <v>723</v>
       </c>
       <c r="J57">
-        <f t="shared" si="21"/>
+        <f t="shared" si="32"/>
         <v>1057</v>
       </c>
       <c r="L57">
@@ -5659,37 +5660,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:26">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C58">
-        <f t="shared" ref="C58:J58" si="22">B32+2*C32+D32</f>
+        <f t="shared" ref="C58:J58" si="33">B32+2*C32+D32</f>
         <v>8</v>
       </c>
       <c r="D58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>11</v>
       </c>
       <c r="E58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>4</v>
       </c>
       <c r="F58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>-4</v>
       </c>
       <c r="G58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>-4</v>
       </c>
       <c r="H58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>9</v>
       </c>
       <c r="I58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>50</v>
       </c>
       <c r="J58">
-        <f t="shared" si="22"/>
+        <f t="shared" si="33"/>
         <v>110</v>
       </c>
       <c r="L58">
@@ -5726,37 +5727,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:26">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C59">
-        <f t="shared" ref="C59:J59" si="23">B33+2*C33+D33</f>
+        <f t="shared" ref="C59:J59" si="34">B33+2*C33+D33</f>
         <v>8</v>
       </c>
       <c r="D59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>-1</v>
       </c>
       <c r="E59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>-6</v>
       </c>
       <c r="F59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>-2</v>
       </c>
       <c r="G59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="H59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="I59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="J59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="L59">
@@ -5793,37 +5794,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:26">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C60">
-        <f t="shared" ref="C60:J60" si="24">B34+2*C34+D34</f>
+        <f t="shared" ref="C60:J60" si="35">B34+2*C34+D34</f>
         <v>-24</v>
       </c>
       <c r="D60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>-16</v>
       </c>
       <c r="E60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>3</v>
       </c>
       <c r="F60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>7</v>
       </c>
       <c r="G60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>0</v>
       </c>
       <c r="H60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>1</v>
       </c>
       <c r="I60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>10</v>
       </c>
       <c r="J60">
-        <f t="shared" si="24"/>
+        <f t="shared" si="35"/>
         <v>10</v>
       </c>
       <c r="L60">
@@ -5860,37 +5861,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:26">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C61">
-        <f t="shared" ref="C61:J61" si="25">B35+2*C35+D35</f>
+        <f t="shared" ref="C61:J61" si="36">B35+2*C35+D35</f>
         <v>11</v>
       </c>
       <c r="D61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>12</v>
       </c>
       <c r="E61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>-2</v>
       </c>
       <c r="F61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>-13</v>
       </c>
       <c r="G61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>-9</v>
       </c>
       <c r="H61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>-1</v>
       </c>
       <c r="I61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>5</v>
       </c>
       <c r="J61">
-        <f t="shared" si="25"/>
+        <f t="shared" si="36"/>
         <v>11</v>
       </c>
       <c r="L61">
@@ -5927,37 +5928,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:26">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C62">
-        <f t="shared" ref="C62:J62" si="26">B36+2*C36+D36</f>
+        <f t="shared" ref="C62:J62" si="37">B36+2*C36+D36</f>
         <v>20</v>
       </c>
       <c r="D62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>11</v>
       </c>
       <c r="E62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>-3</v>
       </c>
       <c r="F62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>-2</v>
       </c>
       <c r="G62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>6</v>
       </c>
       <c r="H62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>8</v>
       </c>
       <c r="I62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>2</v>
       </c>
       <c r="J62">
-        <f t="shared" si="26"/>
+        <f t="shared" si="37"/>
         <v>-2</v>
       </c>
       <c r="L62">
@@ -5994,37 +5995,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:26">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C63">
-        <f t="shared" ref="C63:J63" si="27">B37+2*C37+D37</f>
+        <f t="shared" ref="C63:J63" si="38">B37+2*C37+D37</f>
         <v>-4</v>
       </c>
       <c r="D63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>-7</v>
       </c>
       <c r="E63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>-1</v>
       </c>
       <c r="F63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>13</v>
       </c>
       <c r="G63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>11</v>
       </c>
       <c r="H63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>-8</v>
       </c>
       <c r="I63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>-15</v>
       </c>
       <c r="J63">
-        <f t="shared" si="27"/>
+        <f t="shared" si="38"/>
         <v>-7</v>
       </c>
       <c r="L63">
@@ -6061,37 +6062,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:26">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C64">
-        <f t="shared" ref="C64:J64" si="28">B38+2*C38+D38</f>
+        <f t="shared" ref="C64:J64" si="39">B38+2*C38+D38</f>
         <v>-95</v>
       </c>
       <c r="D64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>-52</v>
       </c>
       <c r="E64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>2</v>
       </c>
       <c r="F64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>3</v>
       </c>
       <c r="G64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>-6</v>
       </c>
       <c r="H64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>-8</v>
       </c>
       <c r="I64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>-2</v>
       </c>
       <c r="J64">
-        <f t="shared" si="28"/>
+        <f t="shared" si="39"/>
         <v>2</v>
       </c>
       <c r="L64">
@@ -6128,37 +6129,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="3:23">
+    <row r="65" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C65">
-        <f t="shared" ref="C65:J65" si="29">B39+2*C39+D39</f>
+        <f t="shared" ref="C65:J65" si="40">B39+2*C39+D39</f>
         <v>-321</v>
       </c>
       <c r="D65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>-201</v>
       </c>
       <c r="E65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>-18</v>
       </c>
       <c r="F65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>6</v>
       </c>
       <c r="G65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>0</v>
       </c>
       <c r="H65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>8</v>
       </c>
       <c r="I65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>12</v>
       </c>
       <c r="J65">
-        <f t="shared" si="29"/>
+        <f t="shared" si="40"/>
         <v>6</v>
       </c>
       <c r="L65">
@@ -6195,7 +6196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="3:23">
+    <row r="66" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C66">
         <f>O42+2*P42+Q42</f>
         <v>6</v>
@@ -6213,19 +6214,19 @@
         <v>#REF!</v>
       </c>
       <c r="G66">
-        <f t="shared" ref="C66:J66" si="30">F43+2*G43+H43</f>
+        <f t="shared" ref="G66:J66" si="41">F43+2*G43+H43</f>
         <v>20</v>
       </c>
       <c r="H66">
-        <f t="shared" si="30"/>
+        <f t="shared" si="41"/>
         <v>24</v>
       </c>
       <c r="I66">
-        <f t="shared" si="30"/>
+        <f t="shared" si="41"/>
         <v>28</v>
       </c>
       <c r="J66">
-        <f t="shared" si="30"/>
+        <f t="shared" si="41"/>
         <v>32</v>
       </c>
       <c r="L66">
@@ -6262,7 +6263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="3:23">
+    <row r="67" spans="3:23" x14ac:dyDescent="0.3">
       <c r="L67">
         <v>0</v>
       </c>
@@ -6305,392 +6306,292 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25497145-3A86-48E4-9DF2-62E8FFF1339A}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1">
         <v>0</v>
       </c>
       <c r="C1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E1">
-        <v>0</v>
-      </c>
-      <c r="F1">
-        <v>0</v>
-      </c>
-      <c r="G1">
-        <v>0</v>
-      </c>
-      <c r="H1">
-        <v>0</v>
-      </c>
-      <c r="I1">
-        <v>0</v>
-      </c>
-      <c r="J1">
-        <v>0</v>
-      </c>
-      <c r="K1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>-8</v>
+        <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>-4</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>-1</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <f>SUM(A1:A3)</f>
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <f t="shared" ref="B8:E8" si="0">SUM(B1:B3)</f>
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <f t="shared" ref="A9:E9" si="1">SUM(A2:A4)</f>
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <f t="shared" ref="A10:E10" si="2">SUM(A3:A5)</f>
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <f>A7-C7</f>
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <f t="shared" ref="C13:D13" si="3">B7-D7</f>
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0</v>
+      </c>
+      <c r="B14">
+        <f t="shared" ref="B14:D14" si="4">A8-C8</f>
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="4"/>
         <v>-15</v>
       </c>
-      <c r="H2">
-        <v>-46</v>
-      </c>
-      <c r="I2">
-        <v>-78</v>
-      </c>
-      <c r="J2">
-        <v>-78</v>
-      </c>
-      <c r="K2">
-        <v>-78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3">
-        <v>0</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>-2</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>-10</v>
-      </c>
-      <c r="J3">
-        <v>-10</v>
-      </c>
-      <c r="K3">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4">
-        <v>-3</v>
-      </c>
-      <c r="B4">
-        <v>-2</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>-1</v>
-      </c>
-      <c r="E5">
-        <v>-1</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>-3</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6">
-        <v>0</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>-3</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>-1</v>
-      </c>
-      <c r="J6">
-        <v>-1</v>
-      </c>
-      <c r="K6">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7">
-        <v>-3</v>
-      </c>
-      <c r="B7">
-        <v>-3</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>-2</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8">
-        <v>-2</v>
-      </c>
-      <c r="F8">
-        <v>-3</v>
-      </c>
-      <c r="G8">
-        <v>3</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9">
-        <v>30</v>
-      </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9">
-        <v>-1</v>
-      </c>
-      <c r="D9">
-        <v>-1</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>2</v>
-      </c>
-      <c r="H9">
-        <v>-1</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10">
-        <v>77</v>
-      </c>
-      <c r="B10">
-        <v>34</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>-3</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>2</v>
-      </c>
-      <c r="G10">
-        <v>-2</v>
-      </c>
-      <c r="H10">
-        <v>-1</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11">
-        <v>0</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11">
+      <c r="D14">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>0</v>
+      </c>
+      <c r="B15">
+        <f t="shared" ref="B15:D15" si="5">A9-C9</f>
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="5"/>
+        <v>-15</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>0</v>
+      </c>
+      <c r="B16">
+        <f t="shared" ref="B16:D16" si="6">A10-C10</f>
+        <v>0</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="6"/>
+        <v>-15</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>0</v>
+      </c>
+      <c r="B17">
+        <f t="shared" ref="B17:D17" si="7">A11-C11</f>
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>0</v>
       </c>
     </row>
@@ -6700,317 +6601,317 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6547A-EFD8-417D-949A-61A399398392}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>0</v>
       </c>
       <c r="B1">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E1">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="F1">
-        <v>520</v>
+        <v>0</v>
       </c>
       <c r="G1">
-        <v>328</v>
+        <v>0</v>
       </c>
       <c r="H1">
-        <v>186</v>
+        <v>0</v>
       </c>
       <c r="I1">
-        <v>283</v>
+        <v>0</v>
       </c>
       <c r="J1">
-        <v>316</v>
+        <v>0</v>
       </c>
       <c r="K1">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="E2">
-        <v>256</v>
+        <v>-1</v>
       </c>
       <c r="F2">
-        <v>510</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>258</v>
+        <v>-15</v>
       </c>
       <c r="H2">
-        <v>16</v>
+        <v>-46</v>
       </c>
       <c r="I2">
-        <v>33</v>
+        <v>-78</v>
       </c>
       <c r="J2">
-        <v>40</v>
+        <v>-78</v>
       </c>
       <c r="K2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>-78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0</v>
       </c>
       <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>-2</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>-10</v>
+      </c>
+      <c r="J3">
+        <v>-10</v>
+      </c>
+      <c r="K3">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>-3</v>
+      </c>
+      <c r="B4">
+        <v>-2</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>-1</v>
+      </c>
+      <c r="E5">
+        <v>-1</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>-3</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>-3</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>-1</v>
+      </c>
+      <c r="J6">
+        <v>-1</v>
+      </c>
+      <c r="K6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>-3</v>
+      </c>
+      <c r="B7">
+        <v>-3</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>-2</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>-2</v>
+      </c>
+      <c r="F8">
+        <v>-3</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>30</v>
+      </c>
+      <c r="B9">
         <v>8</v>
       </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>255</v>
-      </c>
-      <c r="F3">
-        <v>510</v>
-      </c>
-      <c r="G3">
-        <v>255</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4">
-        <v>0</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>258</v>
-      </c>
-      <c r="F4">
-        <v>511</v>
-      </c>
-      <c r="G4">
-        <v>258</v>
-      </c>
-      <c r="H4">
-        <v>6</v>
-      </c>
-      <c r="I4">
-        <v>3</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5">
-        <v>0</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>255</v>
-      </c>
-      <c r="F5">
-        <v>510</v>
-      </c>
-      <c r="G5">
-        <v>255</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6">
-        <v>0</v>
-      </c>
-      <c r="B6">
-        <v>10</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>255</v>
-      </c>
-      <c r="F6">
-        <v>512</v>
-      </c>
-      <c r="G6">
-        <v>259</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7">
-        <v>0</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7">
-        <v>260</v>
-      </c>
-      <c r="F7">
-        <v>512</v>
-      </c>
-      <c r="G7">
-        <v>255</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8">
-        <v>0</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>3</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-      <c r="E8">
-        <v>256</v>
-      </c>
-      <c r="F8">
-        <v>510</v>
-      </c>
-      <c r="G8">
-        <v>256</v>
-      </c>
-      <c r="H8">
-        <v>2</v>
-      </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9">
-        <v>0</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
       <c r="C9">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="E9">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>507</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>259</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -7019,30 +6920,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="B10">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="E10">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>512</v>
+        <v>2</v>
       </c>
       <c r="G10">
-        <v>259</v>
+        <v>-2</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -7054,30 +6955,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>0</v>
       </c>
       <c r="B11">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>254</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>509</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -7095,11 +6996,406 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6547A-EFD8-417D-949A-61A399398392}">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>11</v>
+      </c>
+      <c r="C1">
+        <v>4</v>
+      </c>
+      <c r="D1">
+        <v>9</v>
+      </c>
+      <c r="E1">
+        <v>258</v>
+      </c>
+      <c r="F1">
+        <v>520</v>
+      </c>
+      <c r="G1">
+        <v>328</v>
+      </c>
+      <c r="H1">
+        <v>186</v>
+      </c>
+      <c r="I1">
+        <v>283</v>
+      </c>
+      <c r="J1">
+        <v>316</v>
+      </c>
+      <c r="K1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>256</v>
+      </c>
+      <c r="F2">
+        <v>510</v>
+      </c>
+      <c r="G2">
+        <v>258</v>
+      </c>
+      <c r="H2">
+        <v>16</v>
+      </c>
+      <c r="I2">
+        <v>33</v>
+      </c>
+      <c r="J2">
+        <v>40</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>255</v>
+      </c>
+      <c r="F3">
+        <v>510</v>
+      </c>
+      <c r="G3">
+        <v>255</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>258</v>
+      </c>
+      <c r="F4">
+        <v>511</v>
+      </c>
+      <c r="G4">
+        <v>258</v>
+      </c>
+      <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>255</v>
+      </c>
+      <c r="F5">
+        <v>510</v>
+      </c>
+      <c r="G5">
+        <v>255</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>255</v>
+      </c>
+      <c r="F6">
+        <v>512</v>
+      </c>
+      <c r="G6">
+        <v>259</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>260</v>
+      </c>
+      <c r="F7">
+        <v>512</v>
+      </c>
+      <c r="G7">
+        <v>255</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>256</v>
+      </c>
+      <c r="F8">
+        <v>510</v>
+      </c>
+      <c r="G8">
+        <v>256</v>
+      </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9">
+        <v>255</v>
+      </c>
+      <c r="F9">
+        <v>507</v>
+      </c>
+      <c r="G9">
+        <v>259</v>
+      </c>
+      <c r="H9">
+        <v>5</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>0</v>
+      </c>
+      <c r="B10">
+        <v>46</v>
+      </c>
+      <c r="C10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>255</v>
+      </c>
+      <c r="F10">
+        <v>512</v>
+      </c>
+      <c r="G10">
+        <v>259</v>
+      </c>
+      <c r="H10">
+        <v>2</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="B11">
+        <v>146</v>
+      </c>
+      <c r="C11">
+        <v>34</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>254</v>
+      </c>
+      <c r="F11">
+        <v>509</v>
+      </c>
+      <c r="G11">
+        <v>256</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD5BC59-992F-44C7-98EC-5D6431CF3897}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>0</v>
       </c>
@@ -7134,7 +7430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7169,7 +7465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0</v>
       </c>
@@ -7204,7 +7500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>0</v>
       </c>
@@ -7239,7 +7535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0</v>
       </c>
@@ -7274,7 +7570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>0</v>
       </c>
@@ -7309,7 +7605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0</v>
       </c>
@@ -7344,7 +7640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>0</v>
       </c>
@@ -7379,7 +7675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>0</v>
       </c>
@@ -7414,7 +7710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>0</v>
       </c>
@@ -7449,7 +7745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>0</v>
       </c>

</xml_diff>